<commit_message>
AWS connect and deployed
</commit_message>
<xml_diff>
--- a/templates/eml_metadata_from_sample.xlsx
+++ b/templates/eml_metadata_from_sample.xlsx
@@ -7,12 +7,15 @@
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="creators" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="personnel" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="associated_parties" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
   <si>
     <t xml:space="preserve">Field</t>
   </si>
@@ -36,6 +39,7 @@
   </si>
   <si>
     <t xml:space="preserve">This dataset contains environmental DNA (eDNA) metabarcoding data generated through Minderoo OceanOmics Centre at UWA research projects. The dataset provides information on biological samples collected from marine environments, including sampling locations, collection details, molecular processing, and taxonomic information derived from DNA sequencing. These data support the study of marine biodiversity, species distributions, and environmental monitoring using eDNA approaches. The dataset has been processed and quality checked to support reproducible research and data sharing.
+This dataset reflects the contributions of a large team across sample collection, laboratory processing, and bioinformatic analysis. It was produced by the Minderoo OceanOmics Centre at UWA, in partnership with the Minderoo Foundation, The University of Western Australia (UWA), and the UWA Oceans Institute.
 [This dataset was processed using FAIRe2OBIS.]</t>
   </si>
   <si>
@@ -45,7 +49,7 @@
     <t xml:space="preserve">Keywords</t>
   </si>
   <si>
-    <t xml:space="preserve">metabarcoding, DNA, eDNA, OcOm_2408, OcOm_2408_16SFishD, 16SFishD, OceanOmics, Minderoo, The University of Western Australia, UWA, Minderoo OceanOmics Centre</t>
+    <t xml:space="preserve">metabarcoding, DNA, eDNA, OcOm_2408, OcOm_2408_16SFishD, 16SFishD, OceanOmics, Minderoo, The University of Western Australia, UWA, Minderoo OceanOmics Centre, Fish, Research Data</t>
   </si>
   <si>
     <t xml:space="preserve">Comma-separated</t>
@@ -111,66 +115,45 @@
     <t xml:space="preserve">e.g. AU</t>
   </si>
   <si>
-    <t xml:space="preserve">Creator - given name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creator - surname</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bennett</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creator - position</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bioinformatics Research Officer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creator - email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adam.bennett@uwa.edu.au</t>
+    <t xml:space="preserve">Phone number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0452537745</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional - shared by everyone listed, like the address</t>
   </si>
   <si>
     <t xml:space="preserve">Metadata provider same as creator?</t>
   </si>
   <si>
+    <t xml:space="preserve">TRUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Creator" here means the FIRST row of the separate 'creators' sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metadata provider - given name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only if not same as creator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metadata provider - surname</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metadata provider - position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metadata provider - email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact same as creator?</t>
+  </si>
+  <si>
     <t xml:space="preserve">FALSE</t>
   </si>
   <si>
-    <t xml:space="preserve">Metadata provider - given name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only if not same as creator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metadata provider - surname</t>
-  </si>
-  <si>
-    <t xml:space="preserve">De Jong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metadata provider - position</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Senior Research Fellow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metadata provider - email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">emma.dejong@uwa.edu.au</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact same as creator?</t>
-  </si>
-  <si>
     <t xml:space="preserve">Contact - given name</t>
   </si>
   <si>
@@ -193,48 +176,6 @@
   </si>
   <si>
     <t xml:space="preserve">shannon.corrigan@uwa.edu.au</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Include an associated party?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Associated party - given name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anushka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only if included</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Associated party - surname</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dissanayaka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Associated party - position</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Research Assistant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Associated party - email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anushka.dissanayaka@uwa.edu.au</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Associated party - role</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PUBLISHER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PUBLISHER / AUTHOR / PROCESSOR / EDITOR / REVIEWER / OWNER</t>
   </si>
   <si>
     <t xml:space="preserve">Method steps</t>
@@ -339,16 +280,7 @@
     <t xml:space="preserve">org_country</t>
   </si>
   <si>
-    <t xml:space="preserve">creator_given</t>
-  </si>
-  <si>
-    <t xml:space="preserve">creator_sur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">creator_position</t>
-  </si>
-  <si>
-    <t xml:space="preserve">creator_email</t>
+    <t xml:space="preserve">org_phone</t>
   </si>
   <si>
     <t xml:space="preserve">mp_same</t>
@@ -381,24 +313,6 @@
     <t xml:space="preserve">contact_email</t>
   </si>
   <si>
-    <t xml:space="preserve">ap_include</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ap_given</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ap_sur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ap_position</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ap_email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ap_role</t>
-  </si>
-  <si>
     <t xml:space="preserve">methods</t>
   </si>
   <si>
@@ -424,6 +338,63 @@
   </si>
   <si>
     <t xml:space="preserve">design_desc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Given name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surname</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">raes@minderoo.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minderoo Foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marcelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mayad@minderoo.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POINT_OF_CONTACT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bennett</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adam.bennett@uwa.edu.au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURATOR</t>
   </si>
 </sst>
 </file>
@@ -789,7 +760,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
@@ -803,7 +774,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3">
@@ -817,7 +788,7 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
@@ -831,7 +802,7 @@
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5">
@@ -845,7 +816,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6">
@@ -859,7 +830,7 @@
         <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7">
@@ -873,7 +844,7 @@
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8">
@@ -887,7 +858,7 @@
         <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9">
@@ -901,7 +872,7 @@
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10">
@@ -915,7 +886,7 @@
         <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11">
@@ -929,7 +900,7 @@
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12">
@@ -943,7 +914,7 @@
         <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13">
@@ -954,66 +925,66 @@
         <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="C16" t="s">
         <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18">
@@ -1021,97 +992,97 @@
         <v>42</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>110</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="D19" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="D20" t="s">
-        <v>112</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C22" t="s">
         <v>5</v>
       </c>
       <c r="D22" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="C23" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="D23" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" t="s">
         <v>55</v>
       </c>
-      <c r="C24" t="s">
-        <v>5</v>
-      </c>
       <c r="D24" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25">
@@ -1125,7 +1096,7 @@
         <v>5</v>
       </c>
       <c r="D25" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26">
@@ -1139,7 +1110,7 @@
         <v>5</v>
       </c>
       <c r="D26" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27">
@@ -1147,13 +1118,13 @@
         <v>60</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" t="s">
         <v>61</v>
       </c>
-      <c r="C27" t="s">
-        <v>5</v>
-      </c>
       <c r="D27" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28">
@@ -1164,192 +1135,289 @@
         <v>63</v>
       </c>
       <c r="C28" t="s">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="D28" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="C29" t="s">
         <v>5</v>
       </c>
       <c r="D29" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>68</v>
-      </c>
       <c r="C30" t="s">
         <v>5</v>
       </c>
       <c r="D30" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="C31" t="s">
         <v>5</v>
       </c>
       <c r="D31" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="C32" t="s">
-        <v>73</v>
+        <v>5</v>
       </c>
       <c r="D32" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s">
-        <v>74</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C33" t="s">
-        <v>76</v>
-      </c>
-      <c r="D33" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C34" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s">
-        <v>79</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C35" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s">
-        <v>81</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C36" t="s">
-        <v>82</v>
-      </c>
-      <c r="D36" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="s">
-        <v>83</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C37" t="s">
-        <v>5</v>
-      </c>
-      <c r="D37" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s">
-        <v>85</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C38" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s">
-        <v>87</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C39" t="s">
-        <v>5</v>
-      </c>
-      <c r="D39" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="s">
-        <v>89</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C40" t="s">
-        <v>5</v>
-      </c>
-      <c r="D40" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="s">
-        <v>91</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C41" t="s">
-        <v>5</v>
-      </c>
-      <c r="D41" t="s">
-        <v>133</v>
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="28.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="22.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="24.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="22.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="14.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="14.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="14.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="28.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="24.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="22.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="28.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="24.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="22.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>